<commit_message>
Aggiornata nuovamente lista parti senza cambio di revisione: I condensatori dovevano essere in alluminio non Tantalio
</commit_message>
<xml_diff>
--- a/ESECUTIVI/LP23-325-0_ASSY00_REV01.xlsx
+++ b/ESECUTIVI/LP23-325-0_ASSY00_REV01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documents\Data\Progetti-GIT\HW\PCB-23-325\ESECUTIVI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48131848-C7AC-41B6-A696-544530BE8734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7479B7E-BE17-4536-B2C0-61B1C78BA29A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C5BBDCFD-CE99-4596-997B-437B9C27DA5F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{C5BBDCFD-CE99-4596-997B-437B9C27DA5F}"/>
   </bookViews>
   <sheets>
     <sheet name="23-325-0-ASSY00_REV01" sheetId="1" r:id="rId1"/>
@@ -216,9 +216,6 @@
     <t>C45</t>
   </si>
   <si>
-    <t>Cond.Elt.Tantalio 35V SIZE C</t>
-  </si>
-  <si>
     <t>22uF/25V</t>
   </si>
   <si>
@@ -1263,20 +1260,6 @@
     <t>Prima emissione</t>
   </si>
   <si>
-    <t>M:647-F931E226KCC</t>
-  </si>
-  <si>
-    <t>TNT SIZE C</t>
-  </si>
-  <si>
-    <t>KYOCERA AVX</t>
-  </si>
-  <si>
-    <t>F931E226KCC
-ALTERNATIVI:
- - T491C226K025AT</t>
-  </si>
-  <si>
     <t>REV01</t>
   </si>
   <si>
@@ -1287,21 +1270,6 @@
   </si>
   <si>
     <t>0</t>
-  </si>
-  <si>
-    <t>06/03/2026</t>
-  </si>
-  <si>
-    <t>TNT SIZE B</t>
-  </si>
-  <si>
-    <t>TCJB106M035R0200</t>
-  </si>
-  <si>
-    <t>Cond.Elt.Tantalio 35V SIZE B</t>
-  </si>
-  <si>
-    <t>M:581-TCJB106M035R</t>
   </si>
   <si>
     <t>M: 512-FDS3672
@@ -1325,17 +1293,47 @@
     </r>
   </si>
   <si>
-    <t>Corretto i seguenti references:
-- C45 -&gt; PN:F931E226KCC (size-C invece che D)
-- C47 -&gt; PN:TCJB106M035R0200 (Size B invece che D)
-- Q1 -&gt; BUK7Y153-100EX</t>
-  </si>
-  <si>
     <t>Q1 FDS3672 in package SOIC8 può comunque essere montato sul piazzolato LFPACK (Power SO8)
 In alternativa è stato comunque inserito il componente in formato LFPAK (BUK7Y153-100EX) o alternativi di pari performances</t>
   </si>
   <si>
     <t>27/06/2024</t>
+  </si>
+  <si>
+    <t>EEEFK1E220R</t>
+  </si>
+  <si>
+    <t>PANASONIC</t>
+  </si>
+  <si>
+    <t>D=5mm</t>
+  </si>
+  <si>
+    <t>M:667-EEE-FK1E220R</t>
+  </si>
+  <si>
+    <t>EEE-FKV100UAR</t>
+  </si>
+  <si>
+    <t>Cond.Elt.Alluminioo 25V SIZE C</t>
+  </si>
+  <si>
+    <t>Cond.Elt.Alluminioo 35V SIZE B</t>
+  </si>
+  <si>
+    <t>M:667-EEE-FKV100UAR</t>
+  </si>
+  <si>
+    <t>D=4mm</t>
+  </si>
+  <si>
+    <t>Corretto i seguenti references:
+- C45 -&gt; PN:EEEFK1E220R (All. size-C )
+- C47 -&gt; PN:EEE-FKV100UAR (All. Size B )
+- Q1 -&gt; BUK7Y153-100EX</t>
+  </si>
+  <si>
+    <t>10/03/2026</t>
   </si>
 </sst>
 </file>
@@ -1861,7 +1859,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1894,18 +1892,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2358,7 +2344,7 @@
         <v>39</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>17</v>
@@ -2431,10 +2417,10 @@
         <v>33</v>
       </c>
       <c r="F5" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>402</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>403</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>34</v>
@@ -2487,16 +2473,16 @@
         <v>42</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>43</v>
       </c>
       <c r="F7" s="9" t="s">
+        <v>403</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>404</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>405</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>21</v>
@@ -2516,10 +2502,10 @@
         <v>7</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>23</v>
@@ -2628,74 +2614,74 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:11" s="15" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="12">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
         <v>11</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="8">
         <v>1</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="E12" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="F12" s="9" t="s">
+        <v>419</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="J12" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="F12" s="13" t="s">
-        <v>415</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>412</v>
-      </c>
-      <c r="H12" s="13" t="s">
-        <v>414</v>
-      </c>
-      <c r="I12" s="14" t="s">
-        <v>413</v>
-      </c>
-      <c r="J12" s="13" t="s">
+      <c r="K12" s="12" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>12</v>
+      </c>
+      <c r="B13" s="8">
+        <v>1</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="K12" s="16" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="12">
-        <v>12</v>
-      </c>
-      <c r="B13" s="12">
-        <v>1</v>
-      </c>
-      <c r="C13" s="13" t="s">
+      <c r="D13" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="F13" s="9" t="s">
         <v>423</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="G13" s="9" t="s">
+        <v>426</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>427</v>
+      </c>
+      <c r="J13" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="F13" s="13" t="s">
-        <v>422</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>424</v>
-      </c>
-      <c r="H13" s="13" t="s">
-        <v>414</v>
-      </c>
-      <c r="I13" s="14" t="s">
-        <v>421</v>
-      </c>
-      <c r="J13" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="K13" s="16" t="s">
-        <v>416</v>
+      <c r="K13" s="12" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -2706,7 +2692,7 @@
         <v>2</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>32</v>
@@ -2716,7 +2702,7 @@
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>34</v>
@@ -2736,16 +2722,16 @@
         <v>1</v>
       </c>
       <c r="C15" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="E15" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="F15" s="9" t="s">
         <v>73</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>74</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>21</v>
@@ -2768,13 +2754,13 @@
         <v>1</v>
       </c>
       <c r="C16" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="E16" s="9" t="s">
         <v>76</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>77</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>34</v>
@@ -2800,26 +2786,26 @@
         <v>2</v>
       </c>
       <c r="C17" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D17" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="E17" s="9" t="s">
         <v>79</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>80</v>
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="H17" s="9" t="s">
         <v>81</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>82</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>25</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -2830,28 +2816,28 @@
         <v>7</v>
       </c>
       <c r="C18" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E18" s="9" t="s">
+      <c r="F18" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="G18" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="G18" s="9" t="s">
-        <v>87</v>
-      </c>
       <c r="H18" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I18" s="10" t="s">
         <v>25</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -2862,28 +2848,28 @@
         <v>1</v>
       </c>
       <c r="C19" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D19" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E19" s="9" t="s">
+      <c r="F19" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="G19" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="G19" s="9" t="s">
-        <v>91</v>
-      </c>
       <c r="H19" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I19" s="10" t="s">
         <v>25</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -2894,24 +2880,24 @@
         <v>1</v>
       </c>
       <c r="C20" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="E20" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>94</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H20" s="9"/>
       <c r="I20" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="J20" s="9" t="s">
         <v>96</v>
-      </c>
-      <c r="J20" s="9" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -2922,26 +2908,26 @@
         <v>1</v>
       </c>
       <c r="C21" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="E21" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="H21" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="I21" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="I21" s="10" t="s">
-        <v>103</v>
-      </c>
       <c r="J21" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="60" x14ac:dyDescent="0.25">
@@ -2952,28 +2938,28 @@
         <v>17</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D22" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E22" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="F22" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G22" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="F22" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="G22" s="9" t="s">
+      <c r="H22" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="I22" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="J22" s="9" t="s">
         <v>108</v>
-      </c>
-      <c r="J22" s="9" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -2984,26 +2970,26 @@
         <v>1</v>
       </c>
       <c r="C23" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="E23" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>112</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>113</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>114</v>
       </c>
       <c r="I23" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -3014,26 +3000,26 @@
         <v>1</v>
       </c>
       <c r="C24" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="E24" s="9" t="s">
         <v>117</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>118</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="H24" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="I24" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="J24" s="9" t="s">
         <v>120</v>
-      </c>
-      <c r="I24" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="J24" s="9" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -3044,26 +3030,26 @@
         <v>1</v>
       </c>
       <c r="C25" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="E25" s="9" t="s">
         <v>123</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>124</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="I25" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="J25" s="9" t="s">
         <v>126</v>
-      </c>
-      <c r="I25" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="J25" s="9" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -3074,26 +3060,26 @@
         <v>1</v>
       </c>
       <c r="C26" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="D26" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="E26" s="9" t="s">
         <v>129</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>130</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="H26" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="I26" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="J26" s="9" t="s">
         <v>132</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="J26" s="9" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -3104,26 +3090,26 @@
         <v>1</v>
       </c>
       <c r="C27" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D27" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="E27" s="9" t="s">
         <v>135</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>136</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="H27" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="I27" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="I27" s="10" t="s">
+      <c r="J27" s="9" t="s">
         <v>139</v>
-      </c>
-      <c r="J27" s="9" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -3134,26 +3120,26 @@
         <v>1</v>
       </c>
       <c r="C28" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="D28" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="E28" s="9" t="s">
         <v>142</v>
-      </c>
-      <c r="E28" s="9" t="s">
-        <v>143</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="I28" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="J28" s="9" t="s">
         <v>144</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="J28" s="9" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -3164,26 +3150,26 @@
         <v>1</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D29" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E29" s="9" t="s">
         <v>135</v>
-      </c>
-      <c r="E29" s="9" t="s">
-        <v>136</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="H29" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="H29" s="9" t="s">
+      <c r="I29" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="I29" s="10" t="s">
-        <v>139</v>
-      </c>
       <c r="J29" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
@@ -3194,26 +3180,26 @@
         <v>1</v>
       </c>
       <c r="C30" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="D30" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="E30" s="9" t="s">
         <v>148</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>149</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I30" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J30" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -3224,26 +3210,26 @@
         <v>1</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D31" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E31" s="9" t="s">
         <v>135</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>136</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>137</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>138</v>
       </c>
       <c r="I31" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J31" s="9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -3254,10 +3240,10 @@
         <v>1</v>
       </c>
       <c r="C32" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="D32" s="9" t="s">
         <v>154</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>155</v>
       </c>
       <c r="E32" s="10">
         <v>61200621621</v>
@@ -3266,16 +3252,16 @@
         <v>61200621621</v>
       </c>
       <c r="G32" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="H32" s="9" t="s">
         <v>156</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>157</v>
       </c>
       <c r="I32" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J32" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -3286,28 +3272,28 @@
         <v>1</v>
       </c>
       <c r="C33" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="D33" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="E33" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="F33" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="G33" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="F33" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="G33" s="9" t="s">
+      <c r="H33" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="I33" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="J33" s="9" t="s">
         <v>162</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="I33" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="J33" s="9" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -3318,22 +3304,22 @@
         <v>3</v>
       </c>
       <c r="C34" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="D34" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="E34" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="E34" s="9" t="s">
+      <c r="F34" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="F34" s="9" t="s">
+      <c r="G34" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="G34" s="9" t="s">
-        <v>168</v>
-      </c>
       <c r="H34" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I34" s="10" t="s">
         <v>22</v>
@@ -3350,28 +3336,28 @@
         <v>1</v>
       </c>
       <c r="C35" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="D35" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="E35" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="E35" s="9" t="s">
+      <c r="F35" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="G35" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="F35" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="G35" s="9" t="s">
+      <c r="H35" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="I35" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="H35" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="I35" s="10" t="s">
+      <c r="J35" s="9" t="s">
         <v>173</v>
-      </c>
-      <c r="J35" s="9" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -3382,26 +3368,26 @@
         <v>1</v>
       </c>
       <c r="C36" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="D36" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="E36" s="9" t="s">
         <v>176</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>177</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="H36" s="9" t="s">
         <v>178</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>179</v>
       </c>
       <c r="I36" s="10">
         <v>1038</v>
       </c>
       <c r="J36" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -3412,28 +3398,28 @@
         <v>1</v>
       </c>
       <c r="C37" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="D37" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="E37" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="E37" s="9" t="s">
+      <c r="F37" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="F37" s="9" t="s">
+      <c r="G37" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="G37" s="9" t="s">
+      <c r="H37" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="I37" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="H37" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="I37" s="10" t="s">
+      <c r="J37" s="9" t="s">
         <v>186</v>
-      </c>
-      <c r="J37" s="9" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -3444,28 +3430,28 @@
         <v>1</v>
       </c>
       <c r="C38" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="D38" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="E38" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="E38" s="9" t="s">
+      <c r="F38" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="G38" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="F38" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="G38" s="9" t="s">
+      <c r="H38" s="9" t="s">
         <v>191</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>192</v>
       </c>
       <c r="I38" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J38" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -3476,26 +3462,26 @@
         <v>6</v>
       </c>
       <c r="C39" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="D39" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="D39" s="9" t="s">
+      <c r="E39" s="9" t="s">
         <v>195</v>
-      </c>
-      <c r="E39" s="9" t="s">
-        <v>196</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I39" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J39" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="45" x14ac:dyDescent="0.25">
@@ -3506,29 +3492,29 @@
         <v>1</v>
       </c>
       <c r="C40" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="D40" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="D40" s="9" t="s">
-        <v>200</v>
-      </c>
       <c r="E40" s="9" t="s">
-        <v>426</v>
+        <v>416</v>
       </c>
       <c r="F40" s="9"/>
       <c r="G40" s="9" t="s">
-        <v>425</v>
+        <v>415</v>
       </c>
       <c r="H40" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="I40" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="I40" s="10" t="s">
+      <c r="J40" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="J40" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="K40" s="16" t="s">
-        <v>416</v>
+      <c r="K40" s="12" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="75" x14ac:dyDescent="0.25">
@@ -3539,28 +3525,28 @@
         <v>21</v>
       </c>
       <c r="C41" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="D41" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="D41" s="9" t="s">
+      <c r="E41" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="F41" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="G41" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="F41" s="9" t="s">
-        <v>206</v>
-      </c>
-      <c r="G41" s="9" t="s">
+      <c r="H41" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="I41" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="H41" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="I41" s="10" t="s">
-        <v>208</v>
-      </c>
       <c r="J41" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -3571,26 +3557,26 @@
         <v>2</v>
       </c>
       <c r="C42" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="D42" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="E42" s="9" t="s">
         <v>210</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>211</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H42" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="H42" s="9" t="s">
+      <c r="I42" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="J42" s="9" t="s">
         <v>213</v>
-      </c>
-      <c r="I42" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="J42" s="9" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -3601,26 +3587,26 @@
         <v>1</v>
       </c>
       <c r="C43" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="D43" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="E43" s="9" t="s">
         <v>216</v>
-      </c>
-      <c r="E43" s="9" t="s">
-        <v>217</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="I43" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="H43" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="I43" s="10" t="s">
+      <c r="J43" s="9" t="s">
         <v>219</v>
-      </c>
-      <c r="J43" s="9" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
@@ -3631,19 +3617,19 @@
         <v>1</v>
       </c>
       <c r="C44" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="D44" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="D44" s="9" t="s">
+      <c r="E44" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="E44" s="9" t="s">
+      <c r="F44" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="G44" s="9" t="s">
         <v>223</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="G44" s="9" t="s">
-        <v>224</v>
       </c>
       <c r="H44" s="9" t="s">
         <v>34</v>
@@ -3663,17 +3649,17 @@
         <v>3</v>
       </c>
       <c r="C45" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="D45" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="D45" s="9" t="s">
+      <c r="E45" s="9" t="s">
         <v>226</v>
-      </c>
-      <c r="E45" s="9" t="s">
-        <v>227</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H45" s="9" t="s">
         <v>34</v>
@@ -3693,19 +3679,19 @@
         <v>24</v>
       </c>
       <c r="C46" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E46" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="D46" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E46" s="9" t="s">
-        <v>229</v>
-      </c>
       <c r="F46" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H46" s="9" t="s">
         <v>34</v>
@@ -3725,19 +3711,19 @@
         <v>2</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H47" s="9" t="s">
         <v>34</v>
@@ -3757,19 +3743,19 @@
         <v>18</v>
       </c>
       <c r="C48" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E48" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="D48" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E48" s="9" t="s">
-        <v>232</v>
-      </c>
       <c r="F48" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H48" s="9" t="s">
         <v>34</v>
@@ -3789,19 +3775,19 @@
         <v>3</v>
       </c>
       <c r="C49" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="D49" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="D49" s="9" t="s">
+      <c r="E49" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="E49" s="9" t="s">
-        <v>235</v>
-      </c>
       <c r="F49" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H49" s="9" t="s">
         <v>34</v>
@@ -3821,19 +3807,19 @@
         <v>7</v>
       </c>
       <c r="C50" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E50" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="D50" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="E50" s="9" t="s">
-        <v>237</v>
-      </c>
       <c r="F50" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H50" s="9" t="s">
         <v>34</v>
@@ -3853,17 +3839,17 @@
         <v>1</v>
       </c>
       <c r="C51" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E51" s="9" t="s">
         <v>238</v>
-      </c>
-      <c r="D51" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="E51" s="9" t="s">
-        <v>239</v>
       </c>
       <c r="F51" s="9"/>
       <c r="G51" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H51" s="9" t="s">
         <v>40</v>
@@ -3883,19 +3869,19 @@
         <v>1</v>
       </c>
       <c r="C52" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E52" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="D52" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E52" s="9" t="s">
-        <v>241</v>
-      </c>
       <c r="F52" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H52" s="9" t="s">
         <v>34</v>
@@ -3915,19 +3901,19 @@
         <v>1</v>
       </c>
       <c r="C53" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E53" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="D53" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E53" s="9" t="s">
-        <v>243</v>
-      </c>
       <c r="F53" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H53" s="9" t="s">
         <v>34</v>
@@ -3947,19 +3933,19 @@
         <v>3</v>
       </c>
       <c r="C54" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E54" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="D54" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E54" s="9" t="s">
-        <v>245</v>
-      </c>
       <c r="F54" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H54" s="9" t="s">
         <v>34</v>
@@ -3979,19 +3965,19 @@
         <v>5</v>
       </c>
       <c r="C55" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E55" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="D55" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E55" s="9" t="s">
-        <v>247</v>
-      </c>
       <c r="F55" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H55" s="9" t="s">
         <v>34</v>
@@ -4011,19 +3997,19 @@
         <v>17</v>
       </c>
       <c r="C56" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E56" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="D56" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E56" s="9" t="s">
-        <v>249</v>
-      </c>
       <c r="F56" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H56" s="9" t="s">
         <v>34</v>
@@ -4043,19 +4029,19 @@
         <v>6</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H57" s="9" t="s">
         <v>34</v>
@@ -4075,19 +4061,19 @@
         <v>2</v>
       </c>
       <c r="C58" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E58" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="D58" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E58" s="9" t="s">
-        <v>252</v>
-      </c>
       <c r="F58" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H58" s="9" t="s">
         <v>34</v>
@@ -4107,19 +4093,19 @@
         <v>7</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H59" s="9" t="s">
         <v>34</v>
@@ -4139,19 +4125,19 @@
         <v>7</v>
       </c>
       <c r="C60" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E60" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="D60" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E60" s="9" t="s">
-        <v>255</v>
-      </c>
       <c r="F60" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H60" s="9" t="s">
         <v>34</v>
@@ -4171,19 +4157,19 @@
         <v>7</v>
       </c>
       <c r="C61" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E61" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="D61" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E61" s="9" t="s">
-        <v>257</v>
-      </c>
       <c r="F61" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H61" s="9" t="s">
         <v>34</v>
@@ -4203,19 +4189,19 @@
         <v>3</v>
       </c>
       <c r="C62" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E62" s="9" t="s">
         <v>258</v>
       </c>
-      <c r="D62" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="E62" s="9" t="s">
-        <v>259</v>
-      </c>
       <c r="F62" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H62" s="9" t="s">
         <v>34</v>
@@ -4235,19 +4221,19 @@
         <v>1</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H63" s="9" t="s">
         <v>34</v>
@@ -4267,17 +4253,17 @@
         <v>1</v>
       </c>
       <c r="C64" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="D64" s="9" t="s">
         <v>261</v>
-      </c>
-      <c r="D64" s="9" t="s">
-        <v>262</v>
       </c>
       <c r="E64" s="9">
         <v>100</v>
       </c>
       <c r="F64" s="9"/>
       <c r="G64" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H64" s="9" t="s">
         <v>34</v>
@@ -4297,17 +4283,17 @@
         <v>2</v>
       </c>
       <c r="C65" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E65" s="9" t="s">
         <v>263</v>
-      </c>
-      <c r="D65" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="E65" s="9" t="s">
-        <v>264</v>
       </c>
       <c r="F65" s="9"/>
       <c r="G65" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H65" s="9" t="s">
         <v>34</v>
@@ -4327,20 +4313,20 @@
         <v>6</v>
       </c>
       <c r="C66" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="D66" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="D66" s="9" t="s">
+      <c r="E66" s="9" t="s">
         <v>266</v>
-      </c>
-      <c r="E66" s="9" t="s">
-        <v>267</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="H66" s="9" t="s">
         <v>268</v>
-      </c>
-      <c r="H66" s="9" t="s">
-        <v>269</v>
       </c>
       <c r="I66" s="10" t="s">
         <v>55</v>
@@ -4357,19 +4343,19 @@
         <v>12</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H67" s="9" t="s">
         <v>34</v>
@@ -4389,17 +4375,17 @@
         <v>1</v>
       </c>
       <c r="C68" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E68" s="9">
         <v>100</v>
       </c>
       <c r="F68" s="9"/>
       <c r="G68" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H68" s="9" t="s">
         <v>34</v>
@@ -4419,19 +4405,19 @@
         <v>2</v>
       </c>
       <c r="C69" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="D69" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E69" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="D69" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E69" s="9" t="s">
-        <v>273</v>
-      </c>
       <c r="F69" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H69" s="9" t="s">
         <v>34</v>
@@ -4451,19 +4437,19 @@
         <v>2</v>
       </c>
       <c r="C70" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E70" s="9" t="s">
         <v>274</v>
       </c>
-      <c r="D70" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E70" s="9" t="s">
-        <v>275</v>
-      </c>
       <c r="F70" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H70" s="9" t="s">
         <v>34</v>
@@ -4483,19 +4469,19 @@
         <v>2</v>
       </c>
       <c r="C71" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="D71" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E71" s="9" t="s">
         <v>276</v>
       </c>
-      <c r="D71" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E71" s="9" t="s">
-        <v>277</v>
-      </c>
       <c r="F71" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H71" s="9" t="s">
         <v>34</v>
@@ -4515,10 +4501,10 @@
         <v>1</v>
       </c>
       <c r="C72" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E72" s="9">
         <v>680</v>
@@ -4527,7 +4513,7 @@
         <v>34</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H72" s="9" t="s">
         <v>34</v>
@@ -4547,19 +4533,19 @@
         <v>1</v>
       </c>
       <c r="C73" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="D73" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E73" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="D73" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E73" s="9" t="s">
-        <v>280</v>
-      </c>
       <c r="F73" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H73" s="9" t="s">
         <v>34</v>
@@ -4579,19 +4565,19 @@
         <v>1</v>
       </c>
       <c r="C74" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E74" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="D74" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E74" s="9" t="s">
-        <v>282</v>
-      </c>
       <c r="F74" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H74" s="9" t="s">
         <v>34</v>
@@ -4611,19 +4597,19 @@
         <v>1</v>
       </c>
       <c r="C75" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="D75" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E75" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="D75" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E75" s="9" t="s">
-        <v>284</v>
-      </c>
       <c r="F75" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H75" s="9" t="s">
         <v>34</v>
@@ -4643,19 +4629,19 @@
         <v>1</v>
       </c>
       <c r="C76" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E76" s="9" t="s">
         <v>285</v>
       </c>
-      <c r="D76" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="E76" s="9" t="s">
-        <v>286</v>
-      </c>
       <c r="F76" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H76" s="9" t="s">
         <v>34</v>
@@ -4675,19 +4661,19 @@
         <v>1</v>
       </c>
       <c r="C77" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G77" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H77" s="9" t="s">
         <v>34</v>
@@ -4707,19 +4693,19 @@
         <v>2</v>
       </c>
       <c r="C78" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="D78" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E78" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="D78" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="E78" s="9" t="s">
-        <v>289</v>
-      </c>
       <c r="F78" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H78" s="9" t="s">
         <v>34</v>
@@ -4739,26 +4725,26 @@
         <v>6</v>
       </c>
       <c r="C79" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="D79" s="9" t="s">
         <v>290</v>
       </c>
-      <c r="D79" s="9" t="s">
+      <c r="E79" s="9" t="s">
         <v>291</v>
-      </c>
-      <c r="E79" s="9" t="s">
-        <v>292</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I79" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J79" s="9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="45" x14ac:dyDescent="0.25">
@@ -4769,28 +4755,28 @@
         <v>10</v>
       </c>
       <c r="C80" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="D80" s="9" t="s">
         <v>294</v>
       </c>
-      <c r="D80" s="9" t="s">
+      <c r="E80" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="E80" s="9" t="s">
+      <c r="F80" s="9" t="s">
         <v>296</v>
       </c>
-      <c r="F80" s="9" t="s">
+      <c r="G80" s="9" t="s">
         <v>297</v>
-      </c>
-      <c r="G80" s="9" t="s">
-        <v>298</v>
       </c>
       <c r="H80" s="9" t="s">
         <v>40</v>
       </c>
       <c r="I80" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J80" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="81" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -4801,16 +4787,16 @@
         <v>6</v>
       </c>
       <c r="C81" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="E81" s="9" t="s">
         <v>300</v>
       </c>
-      <c r="D81" s="9" t="s">
-        <v>295</v>
-      </c>
-      <c r="E81" s="9" t="s">
-        <v>301</v>
-      </c>
       <c r="F81" s="9" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G81" s="9"/>
       <c r="H81" s="9"/>
@@ -4823,16 +4809,16 @@
       </c>
       <c r="B82" s="8"/>
       <c r="C82" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="D82" s="9" t="s">
         <v>302</v>
       </c>
-      <c r="D82" s="9" t="s">
+      <c r="E82" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="E82" s="9" t="s">
+      <c r="F82" s="9" t="s">
         <v>304</v>
-      </c>
-      <c r="F82" s="9" t="s">
-        <v>305</v>
       </c>
       <c r="G82" s="9"/>
       <c r="H82" s="9"/>
@@ -4847,26 +4833,26 @@
         <v>4</v>
       </c>
       <c r="C83" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="D83" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="E83" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="D83" s="9" t="s">
-        <v>295</v>
-      </c>
-      <c r="E83" s="9" t="s">
-        <v>307</v>
-      </c>
       <c r="F83" s="9" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G83" s="9"/>
       <c r="H83" s="9" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I83" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="J83" s="9" t="s">
         <v>308</v>
-      </c>
-      <c r="J83" s="9" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="84" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -4877,26 +4863,26 @@
         <v>1</v>
       </c>
       <c r="C84" s="9" t="s">
+        <v>309</v>
+      </c>
+      <c r="D84" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="D84" s="9" t="s">
+      <c r="E84" s="9" t="s">
         <v>311</v>
-      </c>
-      <c r="E84" s="9" t="s">
-        <v>312</v>
       </c>
       <c r="F84" s="9"/>
       <c r="G84" s="9" t="s">
+        <v>312</v>
+      </c>
+      <c r="H84" s="9" t="s">
         <v>313</v>
       </c>
-      <c r="H84" s="9" t="s">
+      <c r="I84" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="I84" s="10" t="s">
+      <c r="J84" s="9" t="s">
         <v>315</v>
-      </c>
-      <c r="J84" s="9" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="85" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -4907,26 +4893,26 @@
         <v>1</v>
       </c>
       <c r="C85" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="D85" s="9" t="s">
         <v>319</v>
       </c>
-      <c r="D85" s="9" t="s">
+      <c r="E85" s="9" t="s">
         <v>320</v>
-      </c>
-      <c r="E85" s="9" t="s">
-        <v>321</v>
       </c>
       <c r="F85" s="9"/>
       <c r="G85" s="9" t="s">
+        <v>321</v>
+      </c>
+      <c r="H85" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="I85" s="10" t="s">
         <v>322</v>
       </c>
-      <c r="H85" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="I85" s="10" t="s">
+      <c r="J85" s="9" t="s">
         <v>323</v>
-      </c>
-      <c r="J85" s="9" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
@@ -4937,28 +4923,28 @@
         <v>1</v>
       </c>
       <c r="C86" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="D86" s="9" t="s">
         <v>325</v>
       </c>
-      <c r="D86" s="9" t="s">
+      <c r="E86" s="9" t="s">
         <v>326</v>
       </c>
-      <c r="E86" s="9" t="s">
+      <c r="F86" s="9" t="s">
+        <v>326</v>
+      </c>
+      <c r="G86" s="9" t="s">
         <v>327</v>
       </c>
-      <c r="F86" s="9" t="s">
-        <v>327</v>
-      </c>
-      <c r="G86" s="9" t="s">
+      <c r="H86" s="9" t="s">
         <v>328</v>
       </c>
-      <c r="H86" s="9" t="s">
+      <c r="I86" s="10" t="s">
         <v>329</v>
       </c>
-      <c r="I86" s="10" t="s">
-        <v>330</v>
-      </c>
       <c r="J86" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="87" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -4969,28 +4955,28 @@
         <v>3</v>
       </c>
       <c r="C87" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="D87" s="9" t="s">
         <v>331</v>
       </c>
-      <c r="D87" s="9" t="s">
+      <c r="E87" s="9" t="s">
         <v>332</v>
       </c>
-      <c r="E87" s="9" t="s">
+      <c r="F87" s="9" t="s">
+        <v>332</v>
+      </c>
+      <c r="G87" s="9" t="s">
         <v>333</v>
       </c>
-      <c r="F87" s="9" t="s">
-        <v>333</v>
-      </c>
-      <c r="G87" s="9" t="s">
+      <c r="H87" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="I87" s="10" t="s">
         <v>334</v>
       </c>
-      <c r="H87" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="I87" s="10" t="s">
+      <c r="J87" s="9" t="s">
         <v>335</v>
-      </c>
-      <c r="J87" s="9" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="88" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -5001,28 +4987,28 @@
         <v>8</v>
       </c>
       <c r="C88" s="9" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D88" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="E88" s="9" t="s">
         <v>317</v>
       </c>
-      <c r="E88" s="9" t="s">
-        <v>318</v>
-      </c>
       <c r="F88" s="9" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G88" s="9" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H88" s="9" t="s">
         <v>40</v>
       </c>
       <c r="I88" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="J88" s="9" t="s">
         <v>338</v>
-      </c>
-      <c r="J88" s="9" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
@@ -5033,28 +5019,28 @@
         <v>2</v>
       </c>
       <c r="C89" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="D89" s="9" t="s">
         <v>340</v>
       </c>
-      <c r="D89" s="9" t="s">
+      <c r="E89" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="E89" s="9" t="s">
+      <c r="F89" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="G89" s="9" t="s">
         <v>342</v>
       </c>
-      <c r="F89" s="9" t="s">
-        <v>342</v>
-      </c>
-      <c r="G89" s="9" t="s">
+      <c r="H89" s="9" t="s">
         <v>343</v>
       </c>
-      <c r="H89" s="9" t="s">
+      <c r="I89" s="10" t="s">
         <v>344</v>
       </c>
-      <c r="I89" s="10" t="s">
+      <c r="J89" s="9" t="s">
         <v>345</v>
-      </c>
-      <c r="J89" s="9" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
@@ -5065,26 +5051,26 @@
         <v>1</v>
       </c>
       <c r="C90" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="D90" s="9" t="s">
         <v>347</v>
       </c>
-      <c r="D90" s="9" t="s">
+      <c r="E90" s="9" t="s">
         <v>348</v>
-      </c>
-      <c r="E90" s="9" t="s">
-        <v>349</v>
       </c>
       <c r="F90" s="9"/>
       <c r="G90" s="9" t="s">
+        <v>349</v>
+      </c>
+      <c r="H90" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="I90" s="10" t="s">
         <v>350</v>
       </c>
-      <c r="H90" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="I90" s="10" t="s">
+      <c r="J90" s="9" t="s">
         <v>351</v>
-      </c>
-      <c r="J90" s="9" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
@@ -5095,26 +5081,26 @@
         <v>2</v>
       </c>
       <c r="C91" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="D91" s="9" t="s">
         <v>353</v>
       </c>
-      <c r="D91" s="9" t="s">
+      <c r="E91" s="9" t="s">
         <v>354</v>
-      </c>
-      <c r="E91" s="9" t="s">
-        <v>355</v>
       </c>
       <c r="F91" s="9"/>
       <c r="G91" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="H91" s="9" t="s">
         <v>356</v>
       </c>
-      <c r="H91" s="9" t="s">
+      <c r="I91" s="10" t="s">
         <v>357</v>
       </c>
-      <c r="I91" s="10" t="s">
+      <c r="J91" s="9" t="s">
         <v>358</v>
-      </c>
-      <c r="J91" s="9" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="92" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -5125,26 +5111,26 @@
         <v>1</v>
       </c>
       <c r="C92" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="D92" s="9" t="s">
         <v>360</v>
       </c>
-      <c r="D92" s="9" t="s">
+      <c r="E92" s="9" t="s">
         <v>361</v>
-      </c>
-      <c r="E92" s="9" t="s">
-        <v>362</v>
       </c>
       <c r="F92" s="9"/>
       <c r="G92" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="H92" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="I92" s="10" t="s">
         <v>363</v>
       </c>
-      <c r="H92" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="I92" s="10" t="s">
+      <c r="J92" s="9" t="s">
         <v>364</v>
-      </c>
-      <c r="J92" s="9" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
@@ -5155,28 +5141,28 @@
         <v>1</v>
       </c>
       <c r="C93" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="D93" s="9" t="s">
         <v>366</v>
       </c>
-      <c r="D93" s="9" t="s">
+      <c r="E93" s="9" t="s">
         <v>367</v>
       </c>
-      <c r="E93" s="9" t="s">
+      <c r="F93" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="G93" s="9" t="s">
         <v>368</v>
       </c>
-      <c r="F93" s="9" t="s">
-        <v>368</v>
-      </c>
-      <c r="G93" s="9" t="s">
+      <c r="H93" s="9" t="s">
         <v>369</v>
-      </c>
-      <c r="H93" s="9" t="s">
-        <v>370</v>
       </c>
       <c r="I93" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J93" s="9" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
@@ -5187,28 +5173,28 @@
         <v>1</v>
       </c>
       <c r="C94" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="D94" s="9" t="s">
         <v>372</v>
       </c>
-      <c r="D94" s="9" t="s">
+      <c r="E94" s="9" t="s">
         <v>373</v>
       </c>
-      <c r="E94" s="9" t="s">
+      <c r="F94" s="9" t="s">
         <v>374</v>
       </c>
-      <c r="F94" s="9" t="s">
+      <c r="G94" s="9" t="s">
         <v>375</v>
       </c>
-      <c r="G94" s="9" t="s">
+      <c r="H94" s="9" t="s">
         <v>376</v>
       </c>
-      <c r="H94" s="9" t="s">
+      <c r="I94" s="10" t="s">
         <v>377</v>
       </c>
-      <c r="I94" s="10" t="s">
-        <v>378</v>
-      </c>
       <c r="J94" s="9" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="95" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -5219,26 +5205,26 @@
         <v>2</v>
       </c>
       <c r="C95" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="D95" s="9" t="s">
         <v>379</v>
       </c>
-      <c r="D95" s="9" t="s">
+      <c r="E95" s="9" t="s">
         <v>380</v>
-      </c>
-      <c r="E95" s="9" t="s">
-        <v>381</v>
       </c>
       <c r="F95" s="9"/>
       <c r="G95" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="H95" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="I95" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="J95" s="9" t="s">
         <v>382</v>
-      </c>
-      <c r="H95" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="I95" s="10" t="s">
-        <v>364</v>
-      </c>
-      <c r="J95" s="9" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="96" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -5249,26 +5235,26 @@
         <v>1</v>
       </c>
       <c r="C96" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="D96" s="9" t="s">
         <v>384</v>
       </c>
-      <c r="D96" s="9" t="s">
+      <c r="E96" s="9" t="s">
         <v>385</v>
-      </c>
-      <c r="E96" s="9" t="s">
-        <v>386</v>
       </c>
       <c r="F96" s="9"/>
       <c r="G96" s="9" t="s">
+        <v>386</v>
+      </c>
+      <c r="H96" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="I96" s="10" t="s">
         <v>387</v>
       </c>
-      <c r="H96" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="I96" s="10" t="s">
+      <c r="J96" s="9" t="s">
         <v>388</v>
-      </c>
-      <c r="J96" s="9" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="97" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -5279,28 +5265,28 @@
         <v>1</v>
       </c>
       <c r="C97" s="9" t="s">
+        <v>389</v>
+      </c>
+      <c r="D97" s="9" t="s">
         <v>390</v>
       </c>
-      <c r="D97" s="9" t="s">
+      <c r="E97" s="9" t="s">
         <v>391</v>
       </c>
-      <c r="E97" s="9" t="s">
+      <c r="F97" s="9" t="s">
+        <v>391</v>
+      </c>
+      <c r="G97" s="9" t="s">
         <v>392</v>
       </c>
-      <c r="F97" s="9" t="s">
-        <v>392</v>
-      </c>
-      <c r="G97" s="9" t="s">
+      <c r="H97" s="9" t="s">
         <v>393</v>
       </c>
-      <c r="H97" s="9" t="s">
+      <c r="I97" s="10" t="s">
         <v>394</v>
       </c>
-      <c r="I97" s="10" t="s">
+      <c r="J97" s="9" t="s">
         <v>395</v>
-      </c>
-      <c r="J97" s="9" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
@@ -5354,68 +5340,68 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.42578125" style="17" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" style="17" customWidth="1"/>
-    <col min="3" max="3" width="50.7109375" style="17" customWidth="1"/>
-    <col min="4" max="4" width="104.42578125" style="17" customWidth="1"/>
+    <col min="1" max="1" width="34.42578125" style="13" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" style="13" customWidth="1"/>
+    <col min="4" max="4" width="104.42578125" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="13" t="s">
+        <v>412</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="11" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="16" t="s">
+        <v>407</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>408</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>418</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>414</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="B6" s="13">
+        <v>1</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>428</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>417</v>
-      </c>
-      <c r="B1" s="17" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" s="11" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="18"/>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="20" t="s">
-        <v>408</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>409</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
-        <v>429</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>419</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
-        <v>420</v>
-      </c>
-      <c r="B6" s="17">
-        <v>1</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>427</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>428</v>
       </c>
     </row>
   </sheetData>

</xml_diff>